<commit_message>
add : new password for account AH177000
</commit_message>
<xml_diff>
--- a/Data Files/userSmile.xlsx
+++ b/Data Files/userSmile.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18750" windowHeight="6800"/>
+    <workbookView windowWidth="19200" windowHeight="6800"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>USM</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>AH177000</t>
+  </si>
+  <si>
+    <t>Bpjstk999!</t>
   </si>
   <si>
     <t>AHMAD RIFQIE ILHAM FIRDAUS</t>
@@ -78,7 +81,7 @@
     <numFmt numFmtId="178" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,13 +94,6 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -547,148 +543,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1071,10 +1067,10 @@
         <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add feature to download and validate pdf
</commit_message>
<xml_diff>
--- a/Data Files/userSmile.xlsx
+++ b/Data Files/userSmile.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>USM</t>
   </si>
@@ -90,6 +90,15 @@
   </si>
   <si>
     <t>GAGA SARI HARYANA</t>
+  </si>
+  <si>
+    <t>MU171920</t>
+  </si>
+  <si>
+    <t>Bpjstk@1</t>
+  </si>
+  <si>
+    <t>MUHAMMAD RIFQI HABIBI</t>
   </si>
 </sst>
 </file>
@@ -1031,8 +1040,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="7" outlineLevelCol="2"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="9.63636363636364" customWidth="1"/>
     <col min="2" max="2" width="10.5454545454545" customWidth="1"/>
@@ -1127,7 +1136,21 @@
         <v>20</v>
       </c>
     </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B9" r:id="rId1" display="Bpjstk@1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>

</xml_diff>